<commit_message>
Progress on Restoration LCA including run script for example evaluation, estimated of coefficients for setting f_E from (runscript for this in 3PG-SoNWaL repo), definition of new function C_Sequest_in_trees_RM which runs the 3PG for the restoration model
</commit_message>
<xml_diff>
--- a/Templates/3PG_parms.xlsx
+++ b/Templates/3PG_parms.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob.osullivan\OneDrive - Forest Research\Turbines and trees\CCWoP\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51838F85-971B-4165-B17F-4B8AE66A28BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A0E65CD-CD8C-4DD8-AABE-E407A1EFD054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{80917C0E-276B-4D0A-AABB-87174A7ED0EB}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{80917C0E-276B-4D0A-AABB-87174A7ED0EB}"/>
   </bookViews>
   <sheets>
     <sheet name="3PG_parms" sheetId="1" r:id="rId1"/>
@@ -1219,10 +1219,10 @@
         <v>46</v>
       </c>
       <c r="C12" s="9">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="D12" s="9">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="E12" s="13" t="s">
         <v>10</v>
@@ -1539,20 +1539,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="040d8fff-bbda-40a8-9b47-f12e1f9ca897" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="040d8fff-bbda-40a8-9b47-f12e1f9ca897" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1738,14 +1738,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{356BE792-C4E2-4568-9742-039A4C8C1533}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85C51094-D249-45EC-8CBB-A6A69EFE2E26}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -1757,6 +1749,14 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{356BE792-C4E2-4568-9742-039A4C8C1533}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
3PG and Forestry modules (harvesting and wood product/biofuel handling) added. For this additional templates added: coefficients used in setting f_E and Growth and Yield tables
</commit_message>
<xml_diff>
--- a/Templates/3PG_parms.xlsx
+++ b/Templates/3PG_parms.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob.osullivan\OneDrive - Forest Research\Turbines and trees\CCWoP\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A0E65CD-CD8C-4DD8-AABE-E407A1EFD054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B493BDB0-0AEE-4A89-81A5-D69497118921}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{80917C0E-276B-4D0A-AABB-87174A7ED0EB}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{80917C0E-276B-4D0A-AABB-87174A7ED0EB}"/>
   </bookViews>
   <sheets>
     <sheet name="3PG_parms" sheetId="1" r:id="rId1"/>
@@ -269,7 +269,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="64">
   <si>
     <t>Parameter</t>
   </si>
@@ -558,6 +558,12 @@
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>Rotation length (yr)</t>
+  </si>
+  <si>
+    <t>t_rotation</t>
   </si>
 </sst>
 </file>
@@ -1023,7 +1029,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685DDD56-94F7-4B65-BA2B-53DE80B2AEAB}">
-  <dimension ref="A1:E23"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43.90625" bestFit="1" customWidth="1"/>
@@ -1332,70 +1339,87 @@
       <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
-        <v>51</v>
+      <c r="A20" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="C20" s="1">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="D20" s="1">
-        <v>1</v>
-      </c>
-      <c r="E20" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C21" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="16" t="s">
-        <v>54</v>
+      <c r="A22" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C22" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0</v>
+      </c>
+      <c r="D23" s="1">
+        <v>0</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B24" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C23" s="1">
-        <v>1</v>
-      </c>
-      <c r="D23" s="1">
-        <v>1</v>
-      </c>
-      <c r="E23" s="7" t="s">
+      <c r="C24" s="1">
+        <v>0</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0</v>
+      </c>
+      <c r="E24" s="7" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1407,6 +1431,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40B7B5A0-E4F8-4333-8A1E-B9B54ACF4FB4}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1539,23 +1564,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="040d8fff-bbda-40a8-9b47-f12e1f9ca897" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001FDF64248B42434C9225F7FDC465556A" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="eccd18745d450949b8e194a7b78b3d64">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="040d8fff-bbda-40a8-9b47-f12e1f9ca897" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f1fb4084c4b078bd4d58554299f480bb" ns3:_="">
     <xsd:import namespace="040d8fff-bbda-40a8-9b47-f12e1f9ca897"/>
@@ -1737,31 +1745,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85C51094-D249-45EC-8CBB-A6A69EFE2E26}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="040d8fff-bbda-40a8-9b47-f12e1f9ca897"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{356BE792-C4E2-4568-9742-039A4C8C1533}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="040d8fff-bbda-40a8-9b47-f12e1f9ca897" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F1DE6BD-E5B2-45B3-B5F5-259926E56996}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1777,4 +1778,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{356BE792-C4E2-4568-9742-039A4C8C1533}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85C51094-D249-45EC-8CBB-A6A69EFE2E26}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="040d8fff-bbda-40a8-9b47-f12e1f9ca897"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>